<commit_message>
Freeze academic hierarchy configuration
</commit_message>
<xml_diff>
--- a/admin-upload-templates/admin-bulk-upload-formats.xlsx
+++ b/admin-upload-templates/admin-bulk-upload-formats.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00 Upload Order" sheetId="1" r:id="R32c609a0e909427b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Guide" sheetId="2" r:id="R06875efeaf344fcc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Qualifications" sheetId="3" r:id="R2cc8b0d0529e44c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 Authorities" sheetId="4" r:id="R11a914c41c7445c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 Programmes" sheetId="5" r:id="Rce3f9b8706484472"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Prog Sections" sheetId="6" r:id="R52480b7326d3438e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Subjects" sheetId="7" r:id="R6d8f0b178b7a4f83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Modules" sheetId="8" r:id="Rb07044ef1a064954"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 Chapters" sheetId="9" r:id="Rd1d7ce829ba84ae6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Topics" sheetId="10" r:id="Re4cdb47fe9534f3e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Resource Types" sheetId="11" r:id="R61d0a4a81ec8430d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Resources" sheetId="12" r:id="R3a854218a0624c56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 Flashcards" sheetId="13" r:id="R8a8f4feefa024a19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Questions" sheetId="14" r:id="Rca0c494e4c954569"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 Exam Info" sheetId="15" r:id="Rc8127b5890e1490f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14 User Status" sheetId="16" r:id="R84febba53ee24d04"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15 Entitlements" sheetId="17" r:id="Rf7192bbb1c2b4085"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00 Upload Order" sheetId="1" r:id="R863d0308efce4a5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Guide" sheetId="2" r:id="R3c6f4bb808294aa2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Qualifications" sheetId="3" r:id="R63ac5874a40249aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 Authorities" sheetId="4" r:id="Rb3a0c80059cf4be2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 Programmes" sheetId="5" r:id="Rfc30499662084484"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Prog Sections" sheetId="6" r:id="Rbdf0f5467aa645e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Subjects" sheetId="7" r:id="Re5e55dc114234c98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Modules" sheetId="8" r:id="R6ebf7a38e86d4659"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 Chapters" sheetId="9" r:id="R026a278dbe174a00"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Topics" sheetId="10" r:id="Rffe03a4b7bf84139"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Resource Types" sheetId="11" r:id="R4b6123f3c7d94cbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Resources" sheetId="12" r:id="Rf2583ea244524919"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 Flashcards" sheetId="13" r:id="Rfcb6d1a7d32b463c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Questions" sheetId="14" r:id="Rdd0541162b9c46d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 Exam Info" sheetId="15" r:id="R1b6993a2dfc54b69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14 User Status" sheetId="16" r:id="R3e0e6df888a6474b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15 Entitlements" sheetId="17" r:id="Rcebf3c15d5ba4c39"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -29,7 +29,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="6">
+  <x:fonts count="7">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -63,8 +63,13 @@
       <x:color rgb="FF0F172A"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF0F172A"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -96,8 +101,18 @@
         <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="3">
+  <x:borders count="4">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -127,11 +142,25 @@
         <x:color rgb="FFE2E8F0"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFE2E8F0"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFE2E8F0"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFE2E8F0"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="28">
+  <x:cellXfs count="47">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -190,6 +219,113 @@
     <x:xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -197,13 +333,30 @@
   <x:dxfs count="1">
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF8FAFC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
   </x:dxfs>
 </x:styleSheet>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<xfpb:FeaturePropertyBags xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <xfpb:bag type="Checkbox"/>
+  <xfpb:bag type="XFControls">
+    <xfpb:bagId k="CellControl">0</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplement">
+    <xfpb:bagId k="XFControls">1</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <xfpb:a k="MappedFeaturePropertyBags">
+      <xfpb:bagId>2</xfpb:bagId>
+    </xfpb:a>
+  </xfpb:bag>
+</xfpb:FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -28599,7 +28752,7 @@
     <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="32" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="70" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="66" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -28859,7 +29012,7 @@
         <x:v>See format</x:v>
       </x:c>
       <x:c r="D20" s="15" t="str">
-        <x:v>Use the value described by the upload type and project documentation.</x:v>
+        <x:v>professional_qualification, broker_exam, surveyor_exam, or specialized_diploma_exam.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -28999,7 +29152,7 @@
         <x:v>Required</x:v>
       </x:c>
       <x:c r="D30" s="15" t="str">
-        <x:v>Stable code. Do not reuse it for a different record.</x:v>
+        <x:v>compulsory, compulsory_optional, optional_credit, general_insurance, life_insurance, reinsurance, broker, surveyor, or spl_diploma.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -29195,7 +29348,7 @@
         <x:v>See format</x:v>
       </x:c>
       <x:c r="D44" s="15" t="str">
-        <x:v>Use the value described by the upload type and project documentation.</x:v>
+        <x:v>Choose a suggested value or enter a reviewed custom category containing 2-120 characters.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -30806,11 +30959,11 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="32" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="13.75" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="29.6299991607666" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="48" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="11" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="7.130000114440918" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
@@ -30831,60 +30984,140 @@
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="27"/>
-      <x:c r="B2" s="27"/>
-      <x:c r="C2" s="27"/>
-      <x:c r="D2" s="27"/>
-      <x:c r="E2" s="27"/>
+      <x:c r="A2" s="43" t="str">
+        <x:v>licentiate</x:v>
+      </x:c>
+      <x:c r="B2" s="43" t="str">
+        <x:v>Licentiate Exam Preparation</x:v>
+      </x:c>
+      <x:c r="C2" s="43" t="str">
+        <x:v>III Licentiate examination preparation.</x:v>
+      </x:c>
+      <x:c r="D2" s="43" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E2" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="27"/>
-      <x:c r="B3" s="27"/>
-      <x:c r="C3" s="27"/>
-      <x:c r="D3" s="27"/>
-      <x:c r="E3" s="27"/>
+      <x:c r="A3" s="43" t="str">
+        <x:v>associate</x:v>
+      </x:c>
+      <x:c r="B3" s="43" t="str">
+        <x:v>Associate Exam Preparation</x:v>
+      </x:c>
+      <x:c r="C3" s="43" t="str">
+        <x:v>III Associate examination preparation.</x:v>
+      </x:c>
+      <x:c r="D3" s="43" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E3" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="27"/>
-      <x:c r="B4" s="27"/>
-      <x:c r="C4" s="27"/>
-      <x:c r="D4" s="27"/>
-      <x:c r="E4" s="27"/>
+      <x:c r="A4" s="43" t="str">
+        <x:v>fellowship</x:v>
+      </x:c>
+      <x:c r="B4" s="43" t="str">
+        <x:v>Fellowship Exam Preparation</x:v>
+      </x:c>
+      <x:c r="C4" s="43" t="str">
+        <x:v>III Fellowship examination preparation.</x:v>
+      </x:c>
+      <x:c r="D4" s="43" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E4" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="27"/>
-      <x:c r="B5" s="27"/>
-      <x:c r="C5" s="27"/>
-      <x:c r="D5" s="27"/>
-      <x:c r="E5" s="27"/>
+      <x:c r="A5" s="43" t="str">
+        <x:v>spl_diploma</x:v>
+      </x:c>
+      <x:c r="B5" s="43" t="str">
+        <x:v>Spl. Dip Exam Preparation</x:v>
+      </x:c>
+      <x:c r="C5" s="43" t="str">
+        <x:v>III specialised diploma examination preparation.</x:v>
+      </x:c>
+      <x:c r="D5" s="43" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E5" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="27"/>
-      <x:c r="B6" s="27"/>
-      <x:c r="C6" s="27"/>
-      <x:c r="D6" s="27"/>
-      <x:c r="E6" s="27"/>
+      <x:c r="A6" s="43" t="str">
+        <x:v>surveyor</x:v>
+      </x:c>
+      <x:c r="B6" s="43" t="str">
+        <x:v>Surveyor Exam Preparation</x:v>
+      </x:c>
+      <x:c r="C6" s="43" t="str">
+        <x:v>III Surveyor examination preparation.</x:v>
+      </x:c>
+      <x:c r="D6" s="43" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E6" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="27"/>
-      <x:c r="B7" s="27"/>
-      <x:c r="C7" s="27"/>
-      <x:c r="D7" s="27"/>
-      <x:c r="E7" s="27"/>
+      <x:c r="A7" s="43" t="str">
+        <x:v>direct_broker</x:v>
+      </x:c>
+      <x:c r="B7" s="43" t="str">
+        <x:v>NIA - Direct Broker Exam Preparation</x:v>
+      </x:c>
+      <x:c r="C7" s="43" t="str">
+        <x:v>General, Life and Health Training</x:v>
+      </x:c>
+      <x:c r="D7" s="43" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E7" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="27"/>
-      <x:c r="B8" s="27"/>
-      <x:c r="C8" s="27"/>
-      <x:c r="D8" s="27"/>
-      <x:c r="E8" s="27"/>
+      <x:c r="A8" s="43" t="str">
+        <x:v>reinsurance_broker</x:v>
+      </x:c>
+      <x:c r="B8" s="43" t="str">
+        <x:v>NIA - Reinsurance Broker Exam Preparation</x:v>
+      </x:c>
+      <x:c r="C8" s="43" t="str">
+        <x:v>NIA Reinsurance Broker examination preparation.</x:v>
+      </x:c>
+      <x:c r="D8" s="43" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E8" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="27"/>
-      <x:c r="B9" s="27"/>
-      <x:c r="C9" s="27"/>
-      <x:c r="D9" s="27"/>
-      <x:c r="E9" s="27"/>
+      <x:c r="A9" s="45" t="str">
+        <x:v>composite_broker</x:v>
+      </x:c>
+      <x:c r="B9" s="45" t="str">
+        <x:v>NIA - Composite Broker Exam Preparation</x:v>
+      </x:c>
+      <x:c r="C9" s="45" t="str">
+        <x:v>NIA Composite Broker examination preparation.</x:v>
+      </x:c>
+      <x:c r="D9" s="45" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E9" s="46" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="27"/>
@@ -35150,18 +35383,18 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="17" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="21" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="32" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="22" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="24" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="19" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="16" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="14" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="12.25" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22.6299991607666" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="48" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="19.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="29.25" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="17.5" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="19.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="14.130000114440918" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="11" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="7.130000114440918" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
@@ -35203,116 +35436,280 @@
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="27"/>
-      <x:c r="B2" s="27"/>
-      <x:c r="C2" s="27"/>
-      <x:c r="D2" s="27"/>
-      <x:c r="E2" s="27"/>
-      <x:c r="F2" s="27"/>
-      <x:c r="G2" s="27"/>
-      <x:c r="H2" s="27"/>
-      <x:c r="I2" s="27"/>
-      <x:c r="J2" s="27"/>
-      <x:c r="K2" s="27"/>
-      <x:c r="L2" s="27"/>
+      <x:c r="A2" s="43" t="str">
+        <x:v>iii</x:v>
+      </x:c>
+      <x:c r="B2" s="43" t="str">
+        <x:v>iii_licentiate</x:v>
+      </x:c>
+      <x:c r="C2" s="43" t="str">
+        <x:v>III - Licentiate Exam Preparation</x:v>
+      </x:c>
+      <x:c r="D2" s="43" t="str">
+        <x:v>professional_qualification</x:v>
+      </x:c>
+      <x:c r="E2" s="43" t="str">
+        <x:v>III Licentiate examination preparation.</x:v>
+      </x:c>
+      <x:c r="F2" s="43" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="G2" s="43" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="H2" s="43"/>
+      <x:c r="I2" s="43"/>
+      <x:c r="J2" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K2" s="43" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L2" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="27"/>
-      <x:c r="B3" s="27"/>
-      <x:c r="C3" s="27"/>
-      <x:c r="D3" s="27"/>
-      <x:c r="E3" s="27"/>
-      <x:c r="F3" s="27"/>
-      <x:c r="G3" s="27"/>
-      <x:c r="H3" s="27"/>
-      <x:c r="I3" s="27"/>
-      <x:c r="J3" s="27"/>
-      <x:c r="K3" s="27"/>
-      <x:c r="L3" s="27"/>
+      <x:c r="A3" s="43" t="str">
+        <x:v>iii</x:v>
+      </x:c>
+      <x:c r="B3" s="43" t="str">
+        <x:v>iii_associate</x:v>
+      </x:c>
+      <x:c r="C3" s="43" t="str">
+        <x:v>III - Associate Exam Preparation</x:v>
+      </x:c>
+      <x:c r="D3" s="43" t="str">
+        <x:v>professional_qualification</x:v>
+      </x:c>
+      <x:c r="E3" s="43" t="str">
+        <x:v>III Associate examination preparation.</x:v>
+      </x:c>
+      <x:c r="F3" s="43" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="G3" s="43" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="H3" s="43"/>
+      <x:c r="I3" s="43"/>
+      <x:c r="J3" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K3" s="43" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L3" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="27"/>
-      <x:c r="B4" s="27"/>
-      <x:c r="C4" s="27"/>
-      <x:c r="D4" s="27"/>
-      <x:c r="E4" s="27"/>
-      <x:c r="F4" s="27"/>
-      <x:c r="G4" s="27"/>
-      <x:c r="H4" s="27"/>
-      <x:c r="I4" s="27"/>
-      <x:c r="J4" s="27"/>
-      <x:c r="K4" s="27"/>
-      <x:c r="L4" s="27"/>
+      <x:c r="A4" s="43" t="str">
+        <x:v>iii</x:v>
+      </x:c>
+      <x:c r="B4" s="43" t="str">
+        <x:v>iii_fellowship</x:v>
+      </x:c>
+      <x:c r="C4" s="43" t="str">
+        <x:v>III - Fellowship Exam Preparation</x:v>
+      </x:c>
+      <x:c r="D4" s="43" t="str">
+        <x:v>professional_qualification</x:v>
+      </x:c>
+      <x:c r="E4" s="43" t="str">
+        <x:v>III Fellowship examination preparation.</x:v>
+      </x:c>
+      <x:c r="F4" s="43" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="G4" s="43" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="H4" s="43"/>
+      <x:c r="I4" s="43"/>
+      <x:c r="J4" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K4" s="43" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L4" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="27"/>
-      <x:c r="B5" s="27"/>
-      <x:c r="C5" s="27"/>
-      <x:c r="D5" s="27"/>
-      <x:c r="E5" s="27"/>
-      <x:c r="F5" s="27"/>
-      <x:c r="G5" s="27"/>
-      <x:c r="H5" s="27"/>
-      <x:c r="I5" s="27"/>
-      <x:c r="J5" s="27"/>
-      <x:c r="K5" s="27"/>
-      <x:c r="L5" s="27"/>
+      <x:c r="A5" s="43" t="str">
+        <x:v>iii</x:v>
+      </x:c>
+      <x:c r="B5" s="43" t="str">
+        <x:v>iii_spl_diploma</x:v>
+      </x:c>
+      <x:c r="C5" s="43" t="str">
+        <x:v>III - Spl. Dip Exam Preparation</x:v>
+      </x:c>
+      <x:c r="D5" s="43" t="str">
+        <x:v>specialized_diploma_exam</x:v>
+      </x:c>
+      <x:c r="E5" s="43" t="str">
+        <x:v>III specialised diploma examination preparation.</x:v>
+      </x:c>
+      <x:c r="F5" s="43" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="G5" s="43" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="H5" s="43"/>
+      <x:c r="I5" s="43"/>
+      <x:c r="J5" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K5" s="43" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="L5" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="27"/>
-      <x:c r="B6" s="27"/>
-      <x:c r="C6" s="27"/>
-      <x:c r="D6" s="27"/>
-      <x:c r="E6" s="27"/>
-      <x:c r="F6" s="27"/>
-      <x:c r="G6" s="27"/>
-      <x:c r="H6" s="27"/>
-      <x:c r="I6" s="27"/>
-      <x:c r="J6" s="27"/>
-      <x:c r="K6" s="27"/>
-      <x:c r="L6" s="27"/>
+      <x:c r="A6" s="43" t="str">
+        <x:v>iii</x:v>
+      </x:c>
+      <x:c r="B6" s="43" t="str">
+        <x:v>iii_surveyor</x:v>
+      </x:c>
+      <x:c r="C6" s="43" t="str">
+        <x:v>III Surveyor Exam Preparation</x:v>
+      </x:c>
+      <x:c r="D6" s="43" t="str">
+        <x:v>surveyor_exam</x:v>
+      </x:c>
+      <x:c r="E6" s="43" t="str">
+        <x:v>III Surveyor examination preparation.</x:v>
+      </x:c>
+      <x:c r="F6" s="43" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="G6" s="43" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="H6" s="43"/>
+      <x:c r="I6" s="43"/>
+      <x:c r="J6" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K6" s="43" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="L6" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="27"/>
-      <x:c r="B7" s="27"/>
-      <x:c r="C7" s="27"/>
-      <x:c r="D7" s="27"/>
-      <x:c r="E7" s="27"/>
-      <x:c r="F7" s="27"/>
-      <x:c r="G7" s="27"/>
-      <x:c r="H7" s="27"/>
-      <x:c r="I7" s="27"/>
-      <x:c r="J7" s="27"/>
-      <x:c r="K7" s="27"/>
-      <x:c r="L7" s="27"/>
+      <x:c r="A7" s="43" t="str">
+        <x:v>nia</x:v>
+      </x:c>
+      <x:c r="B7" s="43" t="str">
+        <x:v>nia_direct_general_health</x:v>
+      </x:c>
+      <x:c r="C7" s="43" t="str">
+        <x:v>Direct Broker Training</x:v>
+      </x:c>
+      <x:c r="D7" s="43" t="str">
+        <x:v>broker_exam</x:v>
+      </x:c>
+      <x:c r="E7" s="43" t="str">
+        <x:v>General, Life and Health Training</x:v>
+      </x:c>
+      <x:c r="F7" s="43" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="G7" s="43" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="H7" s="43"/>
+      <x:c r="I7" s="43"/>
+      <x:c r="J7" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K7" s="43" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L7" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="27"/>
-      <x:c r="B8" s="27"/>
-      <x:c r="C8" s="27"/>
-      <x:c r="D8" s="27"/>
-      <x:c r="E8" s="27"/>
-      <x:c r="F8" s="27"/>
-      <x:c r="G8" s="27"/>
-      <x:c r="H8" s="27"/>
-      <x:c r="I8" s="27"/>
-      <x:c r="J8" s="27"/>
-      <x:c r="K8" s="27"/>
-      <x:c r="L8" s="27"/>
+      <x:c r="A8" s="43" t="str">
+        <x:v>nia</x:v>
+      </x:c>
+      <x:c r="B8" s="43" t="str">
+        <x:v>nia_reinsurance_broker</x:v>
+      </x:c>
+      <x:c r="C8" s="43" t="str">
+        <x:v>Reinsurance Broker Training</x:v>
+      </x:c>
+      <x:c r="D8" s="43" t="str">
+        <x:v>broker_exam</x:v>
+      </x:c>
+      <x:c r="E8" s="43" t="str">
+        <x:v>NIA Reinsurance Broker preparation.</x:v>
+      </x:c>
+      <x:c r="F8" s="43" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="G8" s="43" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="H8" s="43"/>
+      <x:c r="I8" s="43"/>
+      <x:c r="J8" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K8" s="43" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L8" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="27"/>
-      <x:c r="B9" s="27"/>
-      <x:c r="C9" s="27"/>
-      <x:c r="D9" s="27"/>
-      <x:c r="E9" s="27"/>
-      <x:c r="F9" s="27"/>
-      <x:c r="G9" s="27"/>
-      <x:c r="H9" s="27"/>
-      <x:c r="I9" s="27"/>
-      <x:c r="J9" s="27"/>
-      <x:c r="K9" s="27"/>
-      <x:c r="L9" s="27"/>
+      <x:c r="A9" s="45" t="str">
+        <x:v>nia</x:v>
+      </x:c>
+      <x:c r="B9" s="45" t="str">
+        <x:v>nia_composite_broker</x:v>
+      </x:c>
+      <x:c r="C9" s="45" t="str">
+        <x:v>Composite Broker Training</x:v>
+      </x:c>
+      <x:c r="D9" s="45" t="str">
+        <x:v>broker_exam</x:v>
+      </x:c>
+      <x:c r="E9" s="45" t="str">
+        <x:v>Combined Direct Broker and Reinsurance Broker preparation.</x:v>
+      </x:c>
+      <x:c r="F9" s="45" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="G9" s="45" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="H9" s="45" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="I9" s="45" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="J9" s="46" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K9" s="45" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L9" s="46" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="27"/>
@@ -38728,14 +39125,14 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="17" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="32" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="18.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="42" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17.5" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="31.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="11" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="7.130000114440918" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
@@ -38765,314 +39162,686 @@
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="27"/>
-      <x:c r="B2" s="27"/>
-      <x:c r="C2" s="27"/>
-      <x:c r="D2" s="27"/>
-      <x:c r="E2" s="27"/>
-      <x:c r="F2" s="27"/>
-      <x:c r="G2" s="27"/>
-      <x:c r="H2" s="27"/>
+      <x:c r="A2" s="43" t="str">
+        <x:v>iii_licentiate</x:v>
+      </x:c>
+      <x:c r="B2" s="43" t="str">
+        <x:v>compulsory</x:v>
+      </x:c>
+      <x:c r="C2" s="43" t="str">
+        <x:v>Compulsory</x:v>
+      </x:c>
+      <x:c r="D2" s="43" t="str">
+        <x:v>Approved InsureGPTE programme section.</x:v>
+      </x:c>
+      <x:c r="E2" s="43"/>
+      <x:c r="F2" s="43"/>
+      <x:c r="G2" s="43" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H2" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="27"/>
-      <x:c r="B3" s="27"/>
-      <x:c r="C3" s="27"/>
-      <x:c r="D3" s="27"/>
-      <x:c r="E3" s="27"/>
-      <x:c r="F3" s="27"/>
-      <x:c r="G3" s="27"/>
-      <x:c r="H3" s="27"/>
+      <x:c r="A3" s="43" t="str">
+        <x:v>iii_licentiate</x:v>
+      </x:c>
+      <x:c r="B3" s="43" t="str">
+        <x:v>compulsory_optional</x:v>
+      </x:c>
+      <x:c r="C3" s="43" t="str">
+        <x:v>Compulsory Optional</x:v>
+      </x:c>
+      <x:c r="D3" s="43" t="str">
+        <x:v>Approved InsureGPTE programme section.</x:v>
+      </x:c>
+      <x:c r="E3" s="43"/>
+      <x:c r="F3" s="43"/>
+      <x:c r="G3" s="43" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H3" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="27"/>
-      <x:c r="B4" s="27"/>
-      <x:c r="C4" s="27"/>
-      <x:c r="D4" s="27"/>
-      <x:c r="E4" s="27"/>
-      <x:c r="F4" s="27"/>
-      <x:c r="G4" s="27"/>
-      <x:c r="H4" s="27"/>
+      <x:c r="A4" s="43" t="str">
+        <x:v>iii_licentiate</x:v>
+      </x:c>
+      <x:c r="B4" s="43" t="str">
+        <x:v>optional_credit</x:v>
+      </x:c>
+      <x:c r="C4" s="43" t="str">
+        <x:v>Optional Credit</x:v>
+      </x:c>
+      <x:c r="D4" s="43" t="str">
+        <x:v>Approved InsureGPTE programme section.</x:v>
+      </x:c>
+      <x:c r="E4" s="43"/>
+      <x:c r="F4" s="43"/>
+      <x:c r="G4" s="43" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H4" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="27"/>
-      <x:c r="B5" s="27"/>
-      <x:c r="C5" s="27"/>
-      <x:c r="D5" s="27"/>
-      <x:c r="E5" s="27"/>
-      <x:c r="F5" s="27"/>
-      <x:c r="G5" s="27"/>
-      <x:c r="H5" s="27"/>
+      <x:c r="A5" s="43" t="str">
+        <x:v>iii_licentiate</x:v>
+      </x:c>
+      <x:c r="B5" s="43" t="str">
+        <x:v>general_insurance</x:v>
+      </x:c>
+      <x:c r="C5" s="43" t="str">
+        <x:v>General Insurance</x:v>
+      </x:c>
+      <x:c r="D5" s="43" t="str">
+        <x:v>Approved InsureGPTE programme section.</x:v>
+      </x:c>
+      <x:c r="E5" s="43"/>
+      <x:c r="F5" s="43"/>
+      <x:c r="G5" s="43" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H5" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="27"/>
-      <x:c r="B6" s="27"/>
-      <x:c r="C6" s="27"/>
-      <x:c r="D6" s="27"/>
-      <x:c r="E6" s="27"/>
-      <x:c r="F6" s="27"/>
-      <x:c r="G6" s="27"/>
-      <x:c r="H6" s="27"/>
+      <x:c r="A6" s="43" t="str">
+        <x:v>iii_licentiate</x:v>
+      </x:c>
+      <x:c r="B6" s="43" t="str">
+        <x:v>life_insurance</x:v>
+      </x:c>
+      <x:c r="C6" s="43" t="str">
+        <x:v>Life Insurance</x:v>
+      </x:c>
+      <x:c r="D6" s="43" t="str">
+        <x:v>Approved InsureGPTE programme section.</x:v>
+      </x:c>
+      <x:c r="E6" s="43"/>
+      <x:c r="F6" s="43"/>
+      <x:c r="G6" s="43" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H6" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="27"/>
-      <x:c r="B7" s="27"/>
-      <x:c r="C7" s="27"/>
-      <x:c r="D7" s="27"/>
-      <x:c r="E7" s="27"/>
-      <x:c r="F7" s="27"/>
-      <x:c r="G7" s="27"/>
-      <x:c r="H7" s="27"/>
+      <x:c r="A7" s="43" t="str">
+        <x:v>iii_associate</x:v>
+      </x:c>
+      <x:c r="B7" s="43" t="str">
+        <x:v>compulsory</x:v>
+      </x:c>
+      <x:c r="C7" s="43" t="str">
+        <x:v>Compulsory</x:v>
+      </x:c>
+      <x:c r="D7" s="43" t="str">
+        <x:v>Approved InsureGPTE programme section.</x:v>
+      </x:c>
+      <x:c r="E7" s="43"/>
+      <x:c r="F7" s="43"/>
+      <x:c r="G7" s="43" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H7" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="27"/>
-      <x:c r="B8" s="27"/>
-      <x:c r="C8" s="27"/>
-      <x:c r="D8" s="27"/>
-      <x:c r="E8" s="27"/>
-      <x:c r="F8" s="27"/>
-      <x:c r="G8" s="27"/>
-      <x:c r="H8" s="27"/>
+      <x:c r="A8" s="43" t="str">
+        <x:v>iii_associate</x:v>
+      </x:c>
+      <x:c r="B8" s="43" t="str">
+        <x:v>compulsory_optional</x:v>
+      </x:c>
+      <x:c r="C8" s="43" t="str">
+        <x:v>Compulsory Optional</x:v>
+      </x:c>
+      <x:c r="D8" s="43" t="str">
+        <x:v>Approved InsureGPTE programme section.</x:v>
+      </x:c>
+      <x:c r="E8" s="43"/>
+      <x:c r="F8" s="43"/>
+      <x:c r="G8" s="43" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H8" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="27"/>
-      <x:c r="B9" s="27"/>
-      <x:c r="C9" s="27"/>
-      <x:c r="D9" s="27"/>
-      <x:c r="E9" s="27"/>
-      <x:c r="F9" s="27"/>
-      <x:c r="G9" s="27"/>
-      <x:c r="H9" s="27"/>
+      <x:c r="A9" s="43" t="str">
+        <x:v>iii_associate</x:v>
+      </x:c>
+      <x:c r="B9" s="43" t="str">
+        <x:v>optional_credit</x:v>
+      </x:c>
+      <x:c r="C9" s="43" t="str">
+        <x:v>Optional Credit</x:v>
+      </x:c>
+      <x:c r="D9" s="43" t="str">
+        <x:v>Approved InsureGPTE programme section.</x:v>
+      </x:c>
+      <x:c r="E9" s="43"/>
+      <x:c r="F9" s="43"/>
+      <x:c r="G9" s="43" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H9" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="27"/>
-      <x:c r="B10" s="27"/>
-      <x:c r="C10" s="27"/>
-      <x:c r="D10" s="27"/>
-      <x:c r="E10" s="27"/>
-      <x:c r="F10" s="27"/>
-      <x:c r="G10" s="27"/>
-      <x:c r="H10" s="27"/>
+      <x:c r="A10" s="43" t="str">
+        <x:v>iii_associate</x:v>
+      </x:c>
+      <x:c r="B10" s="43" t="str">
+        <x:v>general_insurance</x:v>
+      </x:c>
+      <x:c r="C10" s="43" t="str">
+        <x:v>General Insurance</x:v>
+      </x:c>
+      <x:c r="D10" s="43" t="str">
+        <x:v>Approved InsureGPTE programme section.</x:v>
+      </x:c>
+      <x:c r="E10" s="43"/>
+      <x:c r="F10" s="43"/>
+      <x:c r="G10" s="43" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H10" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="27"/>
-      <x:c r="B11" s="27"/>
-      <x:c r="C11" s="27"/>
-      <x:c r="D11" s="27"/>
-      <x:c r="E11" s="27"/>
-      <x:c r="F11" s="27"/>
-      <x:c r="G11" s="27"/>
-      <x:c r="H11" s="27"/>
+      <x:c r="A11" s="43" t="str">
+        <x:v>iii_associate</x:v>
+      </x:c>
+      <x:c r="B11" s="43" t="str">
+        <x:v>life_insurance</x:v>
+      </x:c>
+      <x:c r="C11" s="43" t="str">
+        <x:v>Life Insurance</x:v>
+      </x:c>
+      <x:c r="D11" s="43" t="str">
+        <x:v>Approved InsureGPTE programme section.</x:v>
+      </x:c>
+      <x:c r="E11" s="43"/>
+      <x:c r="F11" s="43"/>
+      <x:c r="G11" s="43" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H11" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="27"/>
-      <x:c r="B12" s="27"/>
-      <x:c r="C12" s="27"/>
-      <x:c r="D12" s="27"/>
-      <x:c r="E12" s="27"/>
-      <x:c r="F12" s="27"/>
-      <x:c r="G12" s="27"/>
-      <x:c r="H12" s="27"/>
+      <x:c r="A12" s="43" t="str">
+        <x:v>iii_fellowship</x:v>
+      </x:c>
+      <x:c r="B12" s="43" t="str">
+        <x:v>compulsory</x:v>
+      </x:c>
+      <x:c r="C12" s="43" t="str">
+        <x:v>Compulsory</x:v>
+      </x:c>
+      <x:c r="D12" s="43" t="str">
+        <x:v>Approved InsureGPTE programme section.</x:v>
+      </x:c>
+      <x:c r="E12" s="43"/>
+      <x:c r="F12" s="43"/>
+      <x:c r="G12" s="43" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H12" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="27"/>
-      <x:c r="B13" s="27"/>
-      <x:c r="C13" s="27"/>
-      <x:c r="D13" s="27"/>
-      <x:c r="E13" s="27"/>
-      <x:c r="F13" s="27"/>
-      <x:c r="G13" s="27"/>
-      <x:c r="H13" s="27"/>
+      <x:c r="A13" s="43" t="str">
+        <x:v>iii_fellowship</x:v>
+      </x:c>
+      <x:c r="B13" s="43" t="str">
+        <x:v>compulsory_optional</x:v>
+      </x:c>
+      <x:c r="C13" s="43" t="str">
+        <x:v>Compulsory Optional</x:v>
+      </x:c>
+      <x:c r="D13" s="43" t="str">
+        <x:v>Approved InsureGPTE programme section.</x:v>
+      </x:c>
+      <x:c r="E13" s="43"/>
+      <x:c r="F13" s="43"/>
+      <x:c r="G13" s="43" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H13" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="27"/>
-      <x:c r="B14" s="27"/>
-      <x:c r="C14" s="27"/>
-      <x:c r="D14" s="27"/>
-      <x:c r="E14" s="27"/>
-      <x:c r="F14" s="27"/>
-      <x:c r="G14" s="27"/>
-      <x:c r="H14" s="27"/>
+      <x:c r="A14" s="43" t="str">
+        <x:v>iii_fellowship</x:v>
+      </x:c>
+      <x:c r="B14" s="43" t="str">
+        <x:v>optional_credit</x:v>
+      </x:c>
+      <x:c r="C14" s="43" t="str">
+        <x:v>Optional Credit</x:v>
+      </x:c>
+      <x:c r="D14" s="43" t="str">
+        <x:v>Approved InsureGPTE programme section.</x:v>
+      </x:c>
+      <x:c r="E14" s="43"/>
+      <x:c r="F14" s="43"/>
+      <x:c r="G14" s="43" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H14" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="27"/>
-      <x:c r="B15" s="27"/>
-      <x:c r="C15" s="27"/>
-      <x:c r="D15" s="27"/>
-      <x:c r="E15" s="27"/>
-      <x:c r="F15" s="27"/>
-      <x:c r="G15" s="27"/>
-      <x:c r="H15" s="27"/>
+      <x:c r="A15" s="43" t="str">
+        <x:v>iii_fellowship</x:v>
+      </x:c>
+      <x:c r="B15" s="43" t="str">
+        <x:v>general_insurance</x:v>
+      </x:c>
+      <x:c r="C15" s="43" t="str">
+        <x:v>General Insurance</x:v>
+      </x:c>
+      <x:c r="D15" s="43" t="str">
+        <x:v>Approved InsureGPTE programme section.</x:v>
+      </x:c>
+      <x:c r="E15" s="43"/>
+      <x:c r="F15" s="43"/>
+      <x:c r="G15" s="43" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H15" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="27"/>
-      <x:c r="B16" s="27"/>
-      <x:c r="C16" s="27"/>
-      <x:c r="D16" s="27"/>
-      <x:c r="E16" s="27"/>
-      <x:c r="F16" s="27"/>
-      <x:c r="G16" s="27"/>
-      <x:c r="H16" s="27"/>
+      <x:c r="A16" s="43" t="str">
+        <x:v>iii_fellowship</x:v>
+      </x:c>
+      <x:c r="B16" s="43" t="str">
+        <x:v>life_insurance</x:v>
+      </x:c>
+      <x:c r="C16" s="43" t="str">
+        <x:v>Life Insurance</x:v>
+      </x:c>
+      <x:c r="D16" s="43" t="str">
+        <x:v>Approved InsureGPTE programme section.</x:v>
+      </x:c>
+      <x:c r="E16" s="43"/>
+      <x:c r="F16" s="43"/>
+      <x:c r="G16" s="43" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H16" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="27"/>
-      <x:c r="B17" s="27"/>
-      <x:c r="C17" s="27"/>
-      <x:c r="D17" s="27"/>
-      <x:c r="E17" s="27"/>
-      <x:c r="F17" s="27"/>
-      <x:c r="G17" s="27"/>
-      <x:c r="H17" s="27"/>
+      <x:c r="A17" s="43" t="str">
+        <x:v>iii_spl_diploma</x:v>
+      </x:c>
+      <x:c r="B17" s="43" t="str">
+        <x:v>compulsory</x:v>
+      </x:c>
+      <x:c r="C17" s="43" t="str">
+        <x:v>Compulsory</x:v>
+      </x:c>
+      <x:c r="D17" s="43" t="str">
+        <x:v>Approved InsureGPTE programme section.</x:v>
+      </x:c>
+      <x:c r="E17" s="43"/>
+      <x:c r="F17" s="43"/>
+      <x:c r="G17" s="43" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H17" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="27"/>
-      <x:c r="B18" s="27"/>
-      <x:c r="C18" s="27"/>
-      <x:c r="D18" s="27"/>
-      <x:c r="E18" s="27"/>
-      <x:c r="F18" s="27"/>
-      <x:c r="G18" s="27"/>
-      <x:c r="H18" s="27"/>
+      <x:c r="A18" s="43" t="str">
+        <x:v>iii_spl_diploma</x:v>
+      </x:c>
+      <x:c r="B18" s="43" t="str">
+        <x:v>spl_diploma</x:v>
+      </x:c>
+      <x:c r="C18" s="43" t="str">
+        <x:v>Spl_Diploma</x:v>
+      </x:c>
+      <x:c r="D18" s="43" t="str">
+        <x:v>Approved InsureGPTE programme section.</x:v>
+      </x:c>
+      <x:c r="E18" s="43"/>
+      <x:c r="F18" s="43"/>
+      <x:c r="G18" s="43" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H18" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="27"/>
-      <x:c r="B19" s="27"/>
-      <x:c r="C19" s="27"/>
-      <x:c r="D19" s="27"/>
-      <x:c r="E19" s="27"/>
-      <x:c r="F19" s="27"/>
-      <x:c r="G19" s="27"/>
-      <x:c r="H19" s="27"/>
+      <x:c r="A19" s="43" t="str">
+        <x:v>iii_surveyor</x:v>
+      </x:c>
+      <x:c r="B19" s="43" t="str">
+        <x:v>compulsory</x:v>
+      </x:c>
+      <x:c r="C19" s="43" t="str">
+        <x:v>Compulsory</x:v>
+      </x:c>
+      <x:c r="D19" s="43" t="str">
+        <x:v>Approved InsureGPTE programme section.</x:v>
+      </x:c>
+      <x:c r="E19" s="43"/>
+      <x:c r="F19" s="43"/>
+      <x:c r="G19" s="43" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H19" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="27"/>
-      <x:c r="B20" s="27"/>
-      <x:c r="C20" s="27"/>
-      <x:c r="D20" s="27"/>
-      <x:c r="E20" s="27"/>
-      <x:c r="F20" s="27"/>
-      <x:c r="G20" s="27"/>
-      <x:c r="H20" s="27"/>
+      <x:c r="A20" s="43" t="str">
+        <x:v>iii_surveyor</x:v>
+      </x:c>
+      <x:c r="B20" s="43" t="str">
+        <x:v>surveyor</x:v>
+      </x:c>
+      <x:c r="C20" s="43" t="str">
+        <x:v>Surveyor</x:v>
+      </x:c>
+      <x:c r="D20" s="43" t="str">
+        <x:v>Approved InsureGPTE programme section.</x:v>
+      </x:c>
+      <x:c r="E20" s="43"/>
+      <x:c r="F20" s="43"/>
+      <x:c r="G20" s="43" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H20" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="27"/>
-      <x:c r="B21" s="27"/>
-      <x:c r="C21" s="27"/>
-      <x:c r="D21" s="27"/>
-      <x:c r="E21" s="27"/>
-      <x:c r="F21" s="27"/>
-      <x:c r="G21" s="27"/>
-      <x:c r="H21" s="27"/>
+      <x:c r="A21" s="43" t="str">
+        <x:v>nia_direct_general_health</x:v>
+      </x:c>
+      <x:c r="B21" s="43" t="str">
+        <x:v>compulsory</x:v>
+      </x:c>
+      <x:c r="C21" s="43" t="str">
+        <x:v>Compulsory</x:v>
+      </x:c>
+      <x:c r="D21" s="43" t="str">
+        <x:v>Approved InsureGPTE programme section.</x:v>
+      </x:c>
+      <x:c r="E21" s="43"/>
+      <x:c r="F21" s="43"/>
+      <x:c r="G21" s="43" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H21" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="27"/>
-      <x:c r="B22" s="27"/>
-      <x:c r="C22" s="27"/>
-      <x:c r="D22" s="27"/>
-      <x:c r="E22" s="27"/>
-      <x:c r="F22" s="27"/>
-      <x:c r="G22" s="27"/>
-      <x:c r="H22" s="27"/>
+      <x:c r="A22" s="43" t="str">
+        <x:v>nia_direct_general_health</x:v>
+      </x:c>
+      <x:c r="B22" s="43" t="str">
+        <x:v>general_insurance</x:v>
+      </x:c>
+      <x:c r="C22" s="43" t="str">
+        <x:v>General Insurance</x:v>
+      </x:c>
+      <x:c r="D22" s="43" t="str">
+        <x:v>Approved InsureGPTE programme section.</x:v>
+      </x:c>
+      <x:c r="E22" s="43"/>
+      <x:c r="F22" s="43"/>
+      <x:c r="G22" s="43" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H22" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="27"/>
-      <x:c r="B23" s="27"/>
-      <x:c r="C23" s="27"/>
-      <x:c r="D23" s="27"/>
-      <x:c r="E23" s="27"/>
-      <x:c r="F23" s="27"/>
-      <x:c r="G23" s="27"/>
-      <x:c r="H23" s="27"/>
+      <x:c r="A23" s="43" t="str">
+        <x:v>nia_direct_general_health</x:v>
+      </x:c>
+      <x:c r="B23" s="43" t="str">
+        <x:v>life_insurance</x:v>
+      </x:c>
+      <x:c r="C23" s="43" t="str">
+        <x:v>Life Insurance</x:v>
+      </x:c>
+      <x:c r="D23" s="43" t="str">
+        <x:v>Approved InsureGPTE programme section.</x:v>
+      </x:c>
+      <x:c r="E23" s="43"/>
+      <x:c r="F23" s="43"/>
+      <x:c r="G23" s="43" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H23" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="27"/>
-      <x:c r="B24" s="27"/>
-      <x:c r="C24" s="27"/>
-      <x:c r="D24" s="27"/>
-      <x:c r="E24" s="27"/>
-      <x:c r="F24" s="27"/>
-      <x:c r="G24" s="27"/>
-      <x:c r="H24" s="27"/>
+      <x:c r="A24" s="43" t="str">
+        <x:v>nia_direct_general_health</x:v>
+      </x:c>
+      <x:c r="B24" s="43" t="str">
+        <x:v>broker</x:v>
+      </x:c>
+      <x:c r="C24" s="43" t="str">
+        <x:v>Broker</x:v>
+      </x:c>
+      <x:c r="D24" s="43" t="str">
+        <x:v>Approved InsureGPTE programme section.</x:v>
+      </x:c>
+      <x:c r="E24" s="43"/>
+      <x:c r="F24" s="43"/>
+      <x:c r="G24" s="43" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H24" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="27"/>
-      <x:c r="B25" s="27"/>
-      <x:c r="C25" s="27"/>
-      <x:c r="D25" s="27"/>
-      <x:c r="E25" s="27"/>
-      <x:c r="F25" s="27"/>
-      <x:c r="G25" s="27"/>
-      <x:c r="H25" s="27"/>
+      <x:c r="A25" s="43" t="str">
+        <x:v>nia_reinsurance_broker</x:v>
+      </x:c>
+      <x:c r="B25" s="43" t="str">
+        <x:v>compulsory</x:v>
+      </x:c>
+      <x:c r="C25" s="43" t="str">
+        <x:v>Compulsory</x:v>
+      </x:c>
+      <x:c r="D25" s="43" t="str">
+        <x:v>Approved InsureGPTE programme section.</x:v>
+      </x:c>
+      <x:c r="E25" s="43"/>
+      <x:c r="F25" s="43"/>
+      <x:c r="G25" s="43" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H25" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="27"/>
-      <x:c r="B26" s="27"/>
-      <x:c r="C26" s="27"/>
-      <x:c r="D26" s="27"/>
-      <x:c r="E26" s="27"/>
-      <x:c r="F26" s="27"/>
-      <x:c r="G26" s="27"/>
-      <x:c r="H26" s="27"/>
+      <x:c r="A26" s="43" t="str">
+        <x:v>nia_reinsurance_broker</x:v>
+      </x:c>
+      <x:c r="B26" s="43" t="str">
+        <x:v>reinsurance</x:v>
+      </x:c>
+      <x:c r="C26" s="43" t="str">
+        <x:v>Reinsurance</x:v>
+      </x:c>
+      <x:c r="D26" s="43" t="str">
+        <x:v>Approved InsureGPTE programme section.</x:v>
+      </x:c>
+      <x:c r="E26" s="43"/>
+      <x:c r="F26" s="43"/>
+      <x:c r="G26" s="43" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H26" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="27"/>
-      <x:c r="B27" s="27"/>
-      <x:c r="C27" s="27"/>
-      <x:c r="D27" s="27"/>
-      <x:c r="E27" s="27"/>
-      <x:c r="F27" s="27"/>
-      <x:c r="G27" s="27"/>
-      <x:c r="H27" s="27"/>
+      <x:c r="A27" s="43" t="str">
+        <x:v>nia_reinsurance_broker</x:v>
+      </x:c>
+      <x:c r="B27" s="43" t="str">
+        <x:v>broker</x:v>
+      </x:c>
+      <x:c r="C27" s="43" t="str">
+        <x:v>Broker</x:v>
+      </x:c>
+      <x:c r="D27" s="43" t="str">
+        <x:v>Approved InsureGPTE programme section.</x:v>
+      </x:c>
+      <x:c r="E27" s="43"/>
+      <x:c r="F27" s="43"/>
+      <x:c r="G27" s="43" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H27" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="27"/>
-      <x:c r="B28" s="27"/>
-      <x:c r="C28" s="27"/>
-      <x:c r="D28" s="27"/>
-      <x:c r="E28" s="27"/>
-      <x:c r="F28" s="27"/>
-      <x:c r="G28" s="27"/>
-      <x:c r="H28" s="27"/>
+      <x:c r="A28" s="43" t="str">
+        <x:v>nia_composite_broker</x:v>
+      </x:c>
+      <x:c r="B28" s="43" t="str">
+        <x:v>compulsory</x:v>
+      </x:c>
+      <x:c r="C28" s="43" t="str">
+        <x:v>Compulsory</x:v>
+      </x:c>
+      <x:c r="D28" s="43" t="str">
+        <x:v>Approved InsureGPTE programme section.</x:v>
+      </x:c>
+      <x:c r="E28" s="43"/>
+      <x:c r="F28" s="43"/>
+      <x:c r="G28" s="43" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H28" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="27"/>
-      <x:c r="B29" s="27"/>
-      <x:c r="C29" s="27"/>
-      <x:c r="D29" s="27"/>
-      <x:c r="E29" s="27"/>
-      <x:c r="F29" s="27"/>
-      <x:c r="G29" s="27"/>
-      <x:c r="H29" s="27"/>
+      <x:c r="A29" s="43" t="str">
+        <x:v>nia_composite_broker</x:v>
+      </x:c>
+      <x:c r="B29" s="43" t="str">
+        <x:v>general_insurance</x:v>
+      </x:c>
+      <x:c r="C29" s="43" t="str">
+        <x:v>General Insurance</x:v>
+      </x:c>
+      <x:c r="D29" s="43" t="str">
+        <x:v>Approved InsureGPTE programme section.</x:v>
+      </x:c>
+      <x:c r="E29" s="43"/>
+      <x:c r="F29" s="43"/>
+      <x:c r="G29" s="43" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H29" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="27"/>
-      <x:c r="B30" s="27"/>
-      <x:c r="C30" s="27"/>
-      <x:c r="D30" s="27"/>
-      <x:c r="E30" s="27"/>
-      <x:c r="F30" s="27"/>
-      <x:c r="G30" s="27"/>
-      <x:c r="H30" s="27"/>
+      <x:c r="A30" s="43" t="str">
+        <x:v>nia_composite_broker</x:v>
+      </x:c>
+      <x:c r="B30" s="43" t="str">
+        <x:v>life_insurance</x:v>
+      </x:c>
+      <x:c r="C30" s="43" t="str">
+        <x:v>Life Insurance</x:v>
+      </x:c>
+      <x:c r="D30" s="43" t="str">
+        <x:v>Approved InsureGPTE programme section.</x:v>
+      </x:c>
+      <x:c r="E30" s="43"/>
+      <x:c r="F30" s="43"/>
+      <x:c r="G30" s="43" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H30" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="27"/>
-      <x:c r="B31" s="27"/>
-      <x:c r="C31" s="27"/>
-      <x:c r="D31" s="27"/>
-      <x:c r="E31" s="27"/>
-      <x:c r="F31" s="27"/>
-      <x:c r="G31" s="27"/>
-      <x:c r="H31" s="27"/>
+      <x:c r="A31" s="43" t="str">
+        <x:v>nia_composite_broker</x:v>
+      </x:c>
+      <x:c r="B31" s="43" t="str">
+        <x:v>reinsurance</x:v>
+      </x:c>
+      <x:c r="C31" s="43" t="str">
+        <x:v>Reinsurance</x:v>
+      </x:c>
+      <x:c r="D31" s="43" t="str">
+        <x:v>Approved InsureGPTE programme section.</x:v>
+      </x:c>
+      <x:c r="E31" s="43"/>
+      <x:c r="F31" s="43"/>
+      <x:c r="G31" s="43" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H31" s="44" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="27"/>
-      <x:c r="B32" s="27"/>
-      <x:c r="C32" s="27"/>
-      <x:c r="D32" s="27"/>
-      <x:c r="E32" s="27"/>
-      <x:c r="F32" s="27"/>
-      <x:c r="G32" s="27"/>
-      <x:c r="H32" s="27"/>
+      <x:c r="A32" s="45" t="str">
+        <x:v>nia_composite_broker</x:v>
+      </x:c>
+      <x:c r="B32" s="45" t="str">
+        <x:v>broker</x:v>
+      </x:c>
+      <x:c r="C32" s="45" t="str">
+        <x:v>Broker</x:v>
+      </x:c>
+      <x:c r="D32" s="45" t="str">
+        <x:v>Approved InsureGPTE programme section.</x:v>
+      </x:c>
+      <x:c r="E32" s="45"/>
+      <x:c r="F32" s="45"/>
+      <x:c r="G32" s="45" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H32" s="46" t="b">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="27"/>
@@ -45602,7 +46371,7 @@
       <x:c r="O251" s="27"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="4">
+  <x:dataValidations count="5">
     <x:dataValidation type="whole" operator="greaterThanOrEqual" sqref="J2:J251">
       <x:formula1>1</x:formula1>
     </x:dataValidation>
@@ -45614,6 +46383,9 @@
     </x:dataValidation>
     <x:dataValidation type="list" sqref="O2:O251">
       <x:formula1>"true,false"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" allowBlank="1" showDropDown="0" sqref="H2:H251">
+      <x:formula1>"General Insurance,Life Insurance,Common (Life &amp; Non-Life),Regulation and Compliance"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Enforce Architecture Version 1.6 hierarchy
</commit_message>
<xml_diff>
--- a/admin-upload-templates/admin-bulk-upload-formats.xlsx
+++ b/admin-upload-templates/admin-bulk-upload-formats.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00 Upload Order" sheetId="1" r:id="R863d0308efce4a5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Guide" sheetId="2" r:id="R3c6f4bb808294aa2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Qualifications" sheetId="3" r:id="R63ac5874a40249aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 Authorities" sheetId="4" r:id="Rb3a0c80059cf4be2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 Programmes" sheetId="5" r:id="Rfc30499662084484"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Prog Sections" sheetId="6" r:id="Rbdf0f5467aa645e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Subjects" sheetId="7" r:id="Re5e55dc114234c98"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Modules" sheetId="8" r:id="R6ebf7a38e86d4659"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 Chapters" sheetId="9" r:id="R026a278dbe174a00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Topics" sheetId="10" r:id="Rffe03a4b7bf84139"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Resource Types" sheetId="11" r:id="R4b6123f3c7d94cbf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Resources" sheetId="12" r:id="Rf2583ea244524919"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 Flashcards" sheetId="13" r:id="Rfcb6d1a7d32b463c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Questions" sheetId="14" r:id="Rdd0541162b9c46d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 Exam Info" sheetId="15" r:id="R1b6993a2dfc54b69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14 User Status" sheetId="16" r:id="R3e0e6df888a6474b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15 Entitlements" sheetId="17" r:id="Rcebf3c15d5ba4c39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00 Upload Order" sheetId="1" r:id="R5b418cf38f044aab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Guide" sheetId="2" r:id="Rafc744f50ba74b7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Qualifications" sheetId="3" r:id="R611e3ac29ba34e0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 Authorities" sheetId="4" r:id="Redacf204f8914805"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 Programmes" sheetId="5" r:id="Re0b6b0ab8c8b4553"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Prog Sections" sheetId="6" r:id="R08b59a8ac5354d06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Subjects" sheetId="7" r:id="R5ebdf24bd0824a2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Modules" sheetId="8" r:id="Rc49c5ba3ca164365"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 Chapters" sheetId="9" r:id="R793b45396dd040c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Topics" sheetId="10" r:id="Rd086d72098044e3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Resource Types" sheetId="11" r:id="R4a220f20ebb14af4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Resources" sheetId="12" r:id="R0064f9821d2b4163"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 Flashcards" sheetId="13" r:id="R8ee6942d971e4437"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Questions" sheetId="14" r:id="R439449d1d57b4aba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 Exam Info" sheetId="15" r:id="Rae0c0230fcf148dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14 User Status" sheetId="16" r:id="R07f86e7daeb5431d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15 Entitlements" sheetId="17" r:id="Rc3ce73a2313149df"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -69,7 +69,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="9">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -94,6 +94,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFECFDF5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -160,7 +165,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="47">
+  <x:cellXfs count="51">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -319,6 +324,28 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
       <x:extLst>
         <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -29348,7 +29375,7 @@
         <x:v>See format</x:v>
       </x:c>
       <x:c r="D44" s="15" t="str">
-        <x:v>Choose a suggested value or enter a reviewed custom category containing 2-120 characters.</x:v>
+        <x:v>Required. Choose exactly one of the four approved Architecture Version 1.6 categories; custom values are not accepted.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -30984,138 +31011,138 @@
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="43" t="str">
+      <x:c r="A2" s="47" t="str">
         <x:v>licentiate</x:v>
       </x:c>
-      <x:c r="B2" s="43" t="str">
+      <x:c r="B2" s="47" t="str">
         <x:v>Licentiate Exam Preparation</x:v>
       </x:c>
-      <x:c r="C2" s="43" t="str">
+      <x:c r="C2" s="47" t="str">
         <x:v>III Licentiate examination preparation.</x:v>
       </x:c>
-      <x:c r="D2" s="43" t="n">
+      <x:c r="D2" s="47" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E2" s="44" t="b">
+      <x:c r="E2" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="43" t="str">
+      <x:c r="A3" s="47" t="str">
         <x:v>associate</x:v>
       </x:c>
-      <x:c r="B3" s="43" t="str">
+      <x:c r="B3" s="47" t="str">
         <x:v>Associate Exam Preparation</x:v>
       </x:c>
-      <x:c r="C3" s="43" t="str">
+      <x:c r="C3" s="47" t="str">
         <x:v>III Associate examination preparation.</x:v>
       </x:c>
-      <x:c r="D3" s="43" t="n">
+      <x:c r="D3" s="47" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="E3" s="44" t="b">
+      <x:c r="E3" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="43" t="str">
+      <x:c r="A4" s="47" t="str">
         <x:v>fellowship</x:v>
       </x:c>
-      <x:c r="B4" s="43" t="str">
+      <x:c r="B4" s="47" t="str">
         <x:v>Fellowship Exam Preparation</x:v>
       </x:c>
-      <x:c r="C4" s="43" t="str">
+      <x:c r="C4" s="47" t="str">
         <x:v>III Fellowship examination preparation.</x:v>
       </x:c>
-      <x:c r="D4" s="43" t="n">
+      <x:c r="D4" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="E4" s="44" t="b">
+      <x:c r="E4" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="43" t="str">
+      <x:c r="A5" s="47" t="str">
         <x:v>spl_diploma</x:v>
       </x:c>
-      <x:c r="B5" s="43" t="str">
+      <x:c r="B5" s="47" t="str">
         <x:v>Spl. Dip Exam Preparation</x:v>
       </x:c>
-      <x:c r="C5" s="43" t="str">
+      <x:c r="C5" s="47" t="str">
         <x:v>III specialised diploma examination preparation.</x:v>
       </x:c>
-      <x:c r="D5" s="43" t="n">
+      <x:c r="D5" s="47" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="E5" s="44" t="b">
+      <x:c r="E5" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="43" t="str">
+      <x:c r="A6" s="47" t="str">
         <x:v>surveyor</x:v>
       </x:c>
-      <x:c r="B6" s="43" t="str">
+      <x:c r="B6" s="47" t="str">
         <x:v>Surveyor Exam Preparation</x:v>
       </x:c>
-      <x:c r="C6" s="43" t="str">
+      <x:c r="C6" s="47" t="str">
         <x:v>III Surveyor examination preparation.</x:v>
       </x:c>
-      <x:c r="D6" s="43" t="n">
+      <x:c r="D6" s="47" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="E6" s="44" t="b">
+      <x:c r="E6" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="43" t="str">
+      <x:c r="A7" s="47" t="str">
         <x:v>direct_broker</x:v>
       </x:c>
-      <x:c r="B7" s="43" t="str">
+      <x:c r="B7" s="47" t="str">
         <x:v>NIA - Direct Broker Exam Preparation</x:v>
       </x:c>
-      <x:c r="C7" s="43" t="str">
+      <x:c r="C7" s="47" t="str">
         <x:v>General, Life and Health Training</x:v>
       </x:c>
-      <x:c r="D7" s="43" t="n">
+      <x:c r="D7" s="47" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="E7" s="44" t="b">
+      <x:c r="E7" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="43" t="str">
+      <x:c r="A8" s="47" t="str">
         <x:v>reinsurance_broker</x:v>
       </x:c>
-      <x:c r="B8" s="43" t="str">
+      <x:c r="B8" s="47" t="str">
         <x:v>NIA - Reinsurance Broker Exam Preparation</x:v>
       </x:c>
-      <x:c r="C8" s="43" t="str">
+      <x:c r="C8" s="47" t="str">
         <x:v>NIA Reinsurance Broker examination preparation.</x:v>
       </x:c>
-      <x:c r="D8" s="43" t="n">
+      <x:c r="D8" s="47" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="E8" s="44" t="b">
+      <x:c r="E8" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="45" t="str">
+      <x:c r="A9" s="49" t="str">
         <x:v>composite_broker</x:v>
       </x:c>
-      <x:c r="B9" s="45" t="str">
+      <x:c r="B9" s="49" t="str">
         <x:v>NIA - Composite Broker Exam Preparation</x:v>
       </x:c>
-      <x:c r="C9" s="45" t="str">
+      <x:c r="C9" s="49" t="str">
         <x:v>NIA Composite Broker examination preparation.</x:v>
       </x:c>
-      <x:c r="D9" s="45" t="n">
+      <x:c r="D9" s="49" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="E9" s="46" t="b">
+      <x:c r="E9" s="50" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -35385,7 +35412,7 @@
   <x:cols>
     <x:col min="1" max="1" width="12.25" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="18.3799991607666" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="22.6299991607666" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="33" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="18.75" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="48" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="19.3799991607666" hidden="0" customWidth="1"/>
@@ -35436,278 +35463,278 @@
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="43" t="str">
+      <x:c r="A2" s="47" t="str">
         <x:v>iii</x:v>
       </x:c>
-      <x:c r="B2" s="43" t="str">
+      <x:c r="B2" s="47" t="str">
         <x:v>iii_licentiate</x:v>
       </x:c>
-      <x:c r="C2" s="43" t="str">
+      <x:c r="C2" s="47" t="str">
         <x:v>III - Licentiate Exam Preparation</x:v>
       </x:c>
-      <x:c r="D2" s="43" t="str">
+      <x:c r="D2" s="47" t="str">
         <x:v>professional_qualification</x:v>
       </x:c>
-      <x:c r="E2" s="43" t="str">
+      <x:c r="E2" s="47" t="str">
         <x:v>III Licentiate examination preparation.</x:v>
       </x:c>
-      <x:c r="F2" s="43" t="n">
+      <x:c r="F2" s="47" t="n">
         <x:v>60</x:v>
       </x:c>
-      <x:c r="G2" s="43" t="n">
+      <x:c r="G2" s="47" t="n">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="H2" s="43"/>
-      <x:c r="I2" s="43"/>
-      <x:c r="J2" s="44" t="b">
+      <x:c r="H2" s="47"/>
+      <x:c r="I2" s="47"/>
+      <x:c r="J2" s="48" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K2" s="43" t="n">
+      <x:c r="K2" s="47" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="L2" s="44" t="b">
+      <x:c r="L2" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="43" t="str">
+      <x:c r="A3" s="47" t="str">
         <x:v>iii</x:v>
       </x:c>
-      <x:c r="B3" s="43" t="str">
+      <x:c r="B3" s="47" t="str">
         <x:v>iii_associate</x:v>
       </x:c>
-      <x:c r="C3" s="43" t="str">
+      <x:c r="C3" s="47" t="str">
         <x:v>III - Associate Exam Preparation</x:v>
       </x:c>
-      <x:c r="D3" s="43" t="str">
+      <x:c r="D3" s="47" t="str">
         <x:v>professional_qualification</x:v>
       </x:c>
-      <x:c r="E3" s="43" t="str">
+      <x:c r="E3" s="47" t="str">
         <x:v>III Associate examination preparation.</x:v>
       </x:c>
-      <x:c r="F3" s="43" t="n">
+      <x:c r="F3" s="47" t="n">
         <x:v>60</x:v>
       </x:c>
-      <x:c r="G3" s="43" t="n">
+      <x:c r="G3" s="47" t="n">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="H3" s="43"/>
-      <x:c r="I3" s="43"/>
-      <x:c r="J3" s="44" t="b">
+      <x:c r="H3" s="47"/>
+      <x:c r="I3" s="47"/>
+      <x:c r="J3" s="48" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K3" s="43" t="n">
+      <x:c r="K3" s="47" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="L3" s="44" t="b">
+      <x:c r="L3" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="43" t="str">
+      <x:c r="A4" s="47" t="str">
         <x:v>iii</x:v>
       </x:c>
-      <x:c r="B4" s="43" t="str">
+      <x:c r="B4" s="47" t="str">
         <x:v>iii_fellowship</x:v>
       </x:c>
-      <x:c r="C4" s="43" t="str">
+      <x:c r="C4" s="47" t="str">
         <x:v>III - Fellowship Exam Preparation</x:v>
       </x:c>
-      <x:c r="D4" s="43" t="str">
+      <x:c r="D4" s="47" t="str">
         <x:v>professional_qualification</x:v>
       </x:c>
-      <x:c r="E4" s="43" t="str">
+      <x:c r="E4" s="47" t="str">
         <x:v>III Fellowship examination preparation.</x:v>
       </x:c>
-      <x:c r="F4" s="43" t="n">
+      <x:c r="F4" s="47" t="n">
         <x:v>60</x:v>
       </x:c>
-      <x:c r="G4" s="43" t="n">
+      <x:c r="G4" s="47" t="n">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="H4" s="43"/>
-      <x:c r="I4" s="43"/>
-      <x:c r="J4" s="44" t="b">
+      <x:c r="H4" s="47"/>
+      <x:c r="I4" s="47"/>
+      <x:c r="J4" s="48" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K4" s="43" t="n">
+      <x:c r="K4" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="L4" s="44" t="b">
+      <x:c r="L4" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="43" t="str">
+      <x:c r="A5" s="47" t="str">
         <x:v>iii</x:v>
       </x:c>
-      <x:c r="B5" s="43" t="str">
+      <x:c r="B5" s="47" t="str">
         <x:v>iii_spl_diploma</x:v>
       </x:c>
-      <x:c r="C5" s="43" t="str">
+      <x:c r="C5" s="47" t="str">
         <x:v>III - Spl. Dip Exam Preparation</x:v>
       </x:c>
-      <x:c r="D5" s="43" t="str">
+      <x:c r="D5" s="47" t="str">
         <x:v>specialized_diploma_exam</x:v>
       </x:c>
-      <x:c r="E5" s="43" t="str">
+      <x:c r="E5" s="47" t="str">
         <x:v>III specialised diploma examination preparation.</x:v>
       </x:c>
-      <x:c r="F5" s="43" t="n">
+      <x:c r="F5" s="47" t="n">
         <x:v>60</x:v>
       </x:c>
-      <x:c r="G5" s="43" t="n">
+      <x:c r="G5" s="47" t="n">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="H5" s="43"/>
-      <x:c r="I5" s="43"/>
-      <x:c r="J5" s="44" t="b">
+      <x:c r="H5" s="47"/>
+      <x:c r="I5" s="47"/>
+      <x:c r="J5" s="48" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K5" s="43" t="n">
+      <x:c r="K5" s="47" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="L5" s="44" t="b">
+      <x:c r="L5" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="43" t="str">
+      <x:c r="A6" s="47" t="str">
         <x:v>iii</x:v>
       </x:c>
-      <x:c r="B6" s="43" t="str">
+      <x:c r="B6" s="47" t="str">
         <x:v>iii_surveyor</x:v>
       </x:c>
-      <x:c r="C6" s="43" t="str">
+      <x:c r="C6" s="47" t="str">
         <x:v>III Surveyor Exam Preparation</x:v>
       </x:c>
-      <x:c r="D6" s="43" t="str">
+      <x:c r="D6" s="47" t="str">
         <x:v>surveyor_exam</x:v>
       </x:c>
-      <x:c r="E6" s="43" t="str">
+      <x:c r="E6" s="47" t="str">
         <x:v>III Surveyor examination preparation.</x:v>
       </x:c>
-      <x:c r="F6" s="43" t="n">
+      <x:c r="F6" s="47" t="n">
         <x:v>60</x:v>
       </x:c>
-      <x:c r="G6" s="43" t="n">
+      <x:c r="G6" s="47" t="n">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="H6" s="43"/>
-      <x:c r="I6" s="43"/>
-      <x:c r="J6" s="44" t="b">
+      <x:c r="H6" s="47"/>
+      <x:c r="I6" s="47"/>
+      <x:c r="J6" s="48" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K6" s="43" t="n">
+      <x:c r="K6" s="47" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="L6" s="44" t="b">
+      <x:c r="L6" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="43" t="str">
+      <x:c r="A7" s="47" t="str">
         <x:v>nia</x:v>
       </x:c>
-      <x:c r="B7" s="43" t="str">
+      <x:c r="B7" s="47" t="str">
         <x:v>nia_direct_general_health</x:v>
       </x:c>
-      <x:c r="C7" s="43" t="str">
-        <x:v>Direct Broker Training</x:v>
-      </x:c>
-      <x:c r="D7" s="43" t="str">
+      <x:c r="C7" s="47" t="str">
+        <x:v>Direct Broker – General, Life and Health Training</x:v>
+      </x:c>
+      <x:c r="D7" s="47" t="str">
         <x:v>broker_exam</x:v>
       </x:c>
-      <x:c r="E7" s="43" t="str">
+      <x:c r="E7" s="47" t="str">
         <x:v>General, Life and Health Training</x:v>
       </x:c>
-      <x:c r="F7" s="43" t="n">
+      <x:c r="F7" s="47" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="G7" s="43" t="n">
+      <x:c r="G7" s="47" t="n">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="H7" s="43"/>
-      <x:c r="I7" s="43"/>
-      <x:c r="J7" s="44" t="b">
+      <x:c r="H7" s="47"/>
+      <x:c r="I7" s="47"/>
+      <x:c r="J7" s="48" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K7" s="43" t="n">
+      <x:c r="K7" s="47" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="L7" s="44" t="b">
+      <x:c r="L7" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="43" t="str">
+      <x:c r="A8" s="47" t="str">
         <x:v>nia</x:v>
       </x:c>
-      <x:c r="B8" s="43" t="str">
+      <x:c r="B8" s="47" t="str">
         <x:v>nia_reinsurance_broker</x:v>
       </x:c>
-      <x:c r="C8" s="43" t="str">
+      <x:c r="C8" s="47" t="str">
         <x:v>Reinsurance Broker Training</x:v>
       </x:c>
-      <x:c r="D8" s="43" t="str">
+      <x:c r="D8" s="47" t="str">
         <x:v>broker_exam</x:v>
       </x:c>
-      <x:c r="E8" s="43" t="str">
+      <x:c r="E8" s="47" t="str">
         <x:v>NIA Reinsurance Broker preparation.</x:v>
       </x:c>
-      <x:c r="F8" s="43" t="n">
+      <x:c r="F8" s="47" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="G8" s="43" t="n">
+      <x:c r="G8" s="47" t="n">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="H8" s="43"/>
-      <x:c r="I8" s="43"/>
-      <x:c r="J8" s="44" t="b">
+      <x:c r="H8" s="47"/>
+      <x:c r="I8" s="47"/>
+      <x:c r="J8" s="48" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K8" s="43" t="n">
+      <x:c r="K8" s="47" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="L8" s="44" t="b">
+      <x:c r="L8" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="45" t="str">
+      <x:c r="A9" s="49" t="str">
         <x:v>nia</x:v>
       </x:c>
-      <x:c r="B9" s="45" t="str">
+      <x:c r="B9" s="49" t="str">
         <x:v>nia_composite_broker</x:v>
       </x:c>
-      <x:c r="C9" s="45" t="str">
+      <x:c r="C9" s="49" t="str">
         <x:v>Composite Broker Training</x:v>
       </x:c>
-      <x:c r="D9" s="45" t="str">
+      <x:c r="D9" s="49" t="str">
         <x:v>broker_exam</x:v>
       </x:c>
-      <x:c r="E9" s="45" t="str">
+      <x:c r="E9" s="49" t="str">
         <x:v>Combined Direct Broker and Reinsurance Broker preparation.</x:v>
       </x:c>
-      <x:c r="F9" s="45" t="n">
+      <x:c r="F9" s="49" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="G9" s="45" t="n">
+      <x:c r="G9" s="49" t="n">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="H9" s="45" t="n">
+      <x:c r="H9" s="49" t="n">
         <x:v>120</x:v>
       </x:c>
-      <x:c r="I9" s="45" t="n">
+      <x:c r="I9" s="49" t="n">
         <x:v>120</x:v>
       </x:c>
-      <x:c r="J9" s="46" t="b">
+      <x:c r="J9" s="50" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K9" s="45" t="n">
+      <x:c r="K9" s="49" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="L9" s="46" t="b">
+      <x:c r="L9" s="50" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -39162,684 +39189,684 @@
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="43" t="str">
+      <x:c r="A2" s="47" t="str">
         <x:v>iii_licentiate</x:v>
       </x:c>
-      <x:c r="B2" s="43" t="str">
+      <x:c r="B2" s="47" t="str">
         <x:v>compulsory</x:v>
       </x:c>
-      <x:c r="C2" s="43" t="str">
+      <x:c r="C2" s="47" t="str">
         <x:v>Compulsory</x:v>
       </x:c>
-      <x:c r="D2" s="43" t="str">
+      <x:c r="D2" s="47" t="str">
         <x:v>Approved InsureGPTE programme section.</x:v>
       </x:c>
-      <x:c r="E2" s="43"/>
-      <x:c r="F2" s="43"/>
-      <x:c r="G2" s="43" t="n">
+      <x:c r="E2" s="47"/>
+      <x:c r="F2" s="47"/>
+      <x:c r="G2" s="47" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H2" s="44" t="b">
+      <x:c r="H2" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="43" t="str">
+      <x:c r="A3" s="47" t="str">
         <x:v>iii_licentiate</x:v>
       </x:c>
-      <x:c r="B3" s="43" t="str">
+      <x:c r="B3" s="47" t="str">
         <x:v>compulsory_optional</x:v>
       </x:c>
-      <x:c r="C3" s="43" t="str">
+      <x:c r="C3" s="47" t="str">
         <x:v>Compulsory Optional</x:v>
       </x:c>
-      <x:c r="D3" s="43" t="str">
+      <x:c r="D3" s="47" t="str">
         <x:v>Approved InsureGPTE programme section.</x:v>
       </x:c>
-      <x:c r="E3" s="43"/>
-      <x:c r="F3" s="43"/>
-      <x:c r="G3" s="43" t="n">
+      <x:c r="E3" s="47"/>
+      <x:c r="F3" s="47"/>
+      <x:c r="G3" s="47" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="H3" s="44" t="b">
+      <x:c r="H3" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="43" t="str">
+      <x:c r="A4" s="47" t="str">
         <x:v>iii_licentiate</x:v>
       </x:c>
-      <x:c r="B4" s="43" t="str">
+      <x:c r="B4" s="47" t="str">
         <x:v>optional_credit</x:v>
       </x:c>
-      <x:c r="C4" s="43" t="str">
+      <x:c r="C4" s="47" t="str">
         <x:v>Optional Credit</x:v>
       </x:c>
-      <x:c r="D4" s="43" t="str">
+      <x:c r="D4" s="47" t="str">
         <x:v>Approved InsureGPTE programme section.</x:v>
       </x:c>
-      <x:c r="E4" s="43"/>
-      <x:c r="F4" s="43"/>
-      <x:c r="G4" s="43" t="n">
+      <x:c r="E4" s="47"/>
+      <x:c r="F4" s="47"/>
+      <x:c r="G4" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="H4" s="44" t="b">
+      <x:c r="H4" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="43" t="str">
+      <x:c r="A5" s="47" t="str">
         <x:v>iii_licentiate</x:v>
       </x:c>
-      <x:c r="B5" s="43" t="str">
+      <x:c r="B5" s="47" t="str">
         <x:v>general_insurance</x:v>
       </x:c>
-      <x:c r="C5" s="43" t="str">
+      <x:c r="C5" s="47" t="str">
         <x:v>General Insurance</x:v>
       </x:c>
-      <x:c r="D5" s="43" t="str">
+      <x:c r="D5" s="47" t="str">
         <x:v>Approved InsureGPTE programme section.</x:v>
       </x:c>
-      <x:c r="E5" s="43"/>
-      <x:c r="F5" s="43"/>
-      <x:c r="G5" s="43" t="n">
+      <x:c r="E5" s="47"/>
+      <x:c r="F5" s="47"/>
+      <x:c r="G5" s="47" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="H5" s="44" t="b">
+      <x:c r="H5" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="43" t="str">
+      <x:c r="A6" s="47" t="str">
         <x:v>iii_licentiate</x:v>
       </x:c>
-      <x:c r="B6" s="43" t="str">
+      <x:c r="B6" s="47" t="str">
         <x:v>life_insurance</x:v>
       </x:c>
-      <x:c r="C6" s="43" t="str">
+      <x:c r="C6" s="47" t="str">
         <x:v>Life Insurance</x:v>
       </x:c>
-      <x:c r="D6" s="43" t="str">
+      <x:c r="D6" s="47" t="str">
         <x:v>Approved InsureGPTE programme section.</x:v>
       </x:c>
-      <x:c r="E6" s="43"/>
-      <x:c r="F6" s="43"/>
-      <x:c r="G6" s="43" t="n">
+      <x:c r="E6" s="47"/>
+      <x:c r="F6" s="47"/>
+      <x:c r="G6" s="47" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="H6" s="44" t="b">
+      <x:c r="H6" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="43" t="str">
+      <x:c r="A7" s="47" t="str">
         <x:v>iii_associate</x:v>
       </x:c>
-      <x:c r="B7" s="43" t="str">
+      <x:c r="B7" s="47" t="str">
         <x:v>compulsory</x:v>
       </x:c>
-      <x:c r="C7" s="43" t="str">
+      <x:c r="C7" s="47" t="str">
         <x:v>Compulsory</x:v>
       </x:c>
-      <x:c r="D7" s="43" t="str">
+      <x:c r="D7" s="47" t="str">
         <x:v>Approved InsureGPTE programme section.</x:v>
       </x:c>
-      <x:c r="E7" s="43"/>
-      <x:c r="F7" s="43"/>
-      <x:c r="G7" s="43" t="n">
+      <x:c r="E7" s="47"/>
+      <x:c r="F7" s="47"/>
+      <x:c r="G7" s="47" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H7" s="44" t="b">
+      <x:c r="H7" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="43" t="str">
+      <x:c r="A8" s="47" t="str">
         <x:v>iii_associate</x:v>
       </x:c>
-      <x:c r="B8" s="43" t="str">
+      <x:c r="B8" s="47" t="str">
         <x:v>compulsory_optional</x:v>
       </x:c>
-      <x:c r="C8" s="43" t="str">
+      <x:c r="C8" s="47" t="str">
         <x:v>Compulsory Optional</x:v>
       </x:c>
-      <x:c r="D8" s="43" t="str">
+      <x:c r="D8" s="47" t="str">
         <x:v>Approved InsureGPTE programme section.</x:v>
       </x:c>
-      <x:c r="E8" s="43"/>
-      <x:c r="F8" s="43"/>
-      <x:c r="G8" s="43" t="n">
+      <x:c r="E8" s="47"/>
+      <x:c r="F8" s="47"/>
+      <x:c r="G8" s="47" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="H8" s="44" t="b">
+      <x:c r="H8" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="43" t="str">
+      <x:c r="A9" s="47" t="str">
         <x:v>iii_associate</x:v>
       </x:c>
-      <x:c r="B9" s="43" t="str">
+      <x:c r="B9" s="47" t="str">
         <x:v>optional_credit</x:v>
       </x:c>
-      <x:c r="C9" s="43" t="str">
+      <x:c r="C9" s="47" t="str">
         <x:v>Optional Credit</x:v>
       </x:c>
-      <x:c r="D9" s="43" t="str">
+      <x:c r="D9" s="47" t="str">
         <x:v>Approved InsureGPTE programme section.</x:v>
       </x:c>
-      <x:c r="E9" s="43"/>
-      <x:c r="F9" s="43"/>
-      <x:c r="G9" s="43" t="n">
+      <x:c r="E9" s="47"/>
+      <x:c r="F9" s="47"/>
+      <x:c r="G9" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="H9" s="44" t="b">
+      <x:c r="H9" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="43" t="str">
+      <x:c r="A10" s="47" t="str">
         <x:v>iii_associate</x:v>
       </x:c>
-      <x:c r="B10" s="43" t="str">
+      <x:c r="B10" s="47" t="str">
         <x:v>general_insurance</x:v>
       </x:c>
-      <x:c r="C10" s="43" t="str">
+      <x:c r="C10" s="47" t="str">
         <x:v>General Insurance</x:v>
       </x:c>
-      <x:c r="D10" s="43" t="str">
+      <x:c r="D10" s="47" t="str">
         <x:v>Approved InsureGPTE programme section.</x:v>
       </x:c>
-      <x:c r="E10" s="43"/>
-      <x:c r="F10" s="43"/>
-      <x:c r="G10" s="43" t="n">
+      <x:c r="E10" s="47"/>
+      <x:c r="F10" s="47"/>
+      <x:c r="G10" s="47" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="H10" s="44" t="b">
+      <x:c r="H10" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="43" t="str">
+      <x:c r="A11" s="47" t="str">
         <x:v>iii_associate</x:v>
       </x:c>
-      <x:c r="B11" s="43" t="str">
+      <x:c r="B11" s="47" t="str">
         <x:v>life_insurance</x:v>
       </x:c>
-      <x:c r="C11" s="43" t="str">
+      <x:c r="C11" s="47" t="str">
         <x:v>Life Insurance</x:v>
       </x:c>
-      <x:c r="D11" s="43" t="str">
+      <x:c r="D11" s="47" t="str">
         <x:v>Approved InsureGPTE programme section.</x:v>
       </x:c>
-      <x:c r="E11" s="43"/>
-      <x:c r="F11" s="43"/>
-      <x:c r="G11" s="43" t="n">
+      <x:c r="E11" s="47"/>
+      <x:c r="F11" s="47"/>
+      <x:c r="G11" s="47" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="H11" s="44" t="b">
+      <x:c r="H11" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="43" t="str">
+      <x:c r="A12" s="47" t="str">
         <x:v>iii_fellowship</x:v>
       </x:c>
-      <x:c r="B12" s="43" t="str">
+      <x:c r="B12" s="47" t="str">
         <x:v>compulsory</x:v>
       </x:c>
-      <x:c r="C12" s="43" t="str">
+      <x:c r="C12" s="47" t="str">
         <x:v>Compulsory</x:v>
       </x:c>
-      <x:c r="D12" s="43" t="str">
+      <x:c r="D12" s="47" t="str">
         <x:v>Approved InsureGPTE programme section.</x:v>
       </x:c>
-      <x:c r="E12" s="43"/>
-      <x:c r="F12" s="43"/>
-      <x:c r="G12" s="43" t="n">
+      <x:c r="E12" s="47"/>
+      <x:c r="F12" s="47"/>
+      <x:c r="G12" s="47" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H12" s="44" t="b">
+      <x:c r="H12" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="43" t="str">
+      <x:c r="A13" s="47" t="str">
         <x:v>iii_fellowship</x:v>
       </x:c>
-      <x:c r="B13" s="43" t="str">
+      <x:c r="B13" s="47" t="str">
         <x:v>compulsory_optional</x:v>
       </x:c>
-      <x:c r="C13" s="43" t="str">
+      <x:c r="C13" s="47" t="str">
         <x:v>Compulsory Optional</x:v>
       </x:c>
-      <x:c r="D13" s="43" t="str">
+      <x:c r="D13" s="47" t="str">
         <x:v>Approved InsureGPTE programme section.</x:v>
       </x:c>
-      <x:c r="E13" s="43"/>
-      <x:c r="F13" s="43"/>
-      <x:c r="G13" s="43" t="n">
+      <x:c r="E13" s="47"/>
+      <x:c r="F13" s="47"/>
+      <x:c r="G13" s="47" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="H13" s="44" t="b">
+      <x:c r="H13" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="43" t="str">
+      <x:c r="A14" s="47" t="str">
         <x:v>iii_fellowship</x:v>
       </x:c>
-      <x:c r="B14" s="43" t="str">
+      <x:c r="B14" s="47" t="str">
         <x:v>optional_credit</x:v>
       </x:c>
-      <x:c r="C14" s="43" t="str">
+      <x:c r="C14" s="47" t="str">
         <x:v>Optional Credit</x:v>
       </x:c>
-      <x:c r="D14" s="43" t="str">
+      <x:c r="D14" s="47" t="str">
         <x:v>Approved InsureGPTE programme section.</x:v>
       </x:c>
-      <x:c r="E14" s="43"/>
-      <x:c r="F14" s="43"/>
-      <x:c r="G14" s="43" t="n">
+      <x:c r="E14" s="47"/>
+      <x:c r="F14" s="47"/>
+      <x:c r="G14" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="H14" s="44" t="b">
+      <x:c r="H14" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="43" t="str">
+      <x:c r="A15" s="47" t="str">
         <x:v>iii_fellowship</x:v>
       </x:c>
-      <x:c r="B15" s="43" t="str">
+      <x:c r="B15" s="47" t="str">
         <x:v>general_insurance</x:v>
       </x:c>
-      <x:c r="C15" s="43" t="str">
+      <x:c r="C15" s="47" t="str">
         <x:v>General Insurance</x:v>
       </x:c>
-      <x:c r="D15" s="43" t="str">
+      <x:c r="D15" s="47" t="str">
         <x:v>Approved InsureGPTE programme section.</x:v>
       </x:c>
-      <x:c r="E15" s="43"/>
-      <x:c r="F15" s="43"/>
-      <x:c r="G15" s="43" t="n">
+      <x:c r="E15" s="47"/>
+      <x:c r="F15" s="47"/>
+      <x:c r="G15" s="47" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="H15" s="44" t="b">
+      <x:c r="H15" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="43" t="str">
+      <x:c r="A16" s="47" t="str">
         <x:v>iii_fellowship</x:v>
       </x:c>
-      <x:c r="B16" s="43" t="str">
+      <x:c r="B16" s="47" t="str">
         <x:v>life_insurance</x:v>
       </x:c>
-      <x:c r="C16" s="43" t="str">
+      <x:c r="C16" s="47" t="str">
         <x:v>Life Insurance</x:v>
       </x:c>
-      <x:c r="D16" s="43" t="str">
+      <x:c r="D16" s="47" t="str">
         <x:v>Approved InsureGPTE programme section.</x:v>
       </x:c>
-      <x:c r="E16" s="43"/>
-      <x:c r="F16" s="43"/>
-      <x:c r="G16" s="43" t="n">
+      <x:c r="E16" s="47"/>
+      <x:c r="F16" s="47"/>
+      <x:c r="G16" s="47" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="H16" s="44" t="b">
+      <x:c r="H16" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="43" t="str">
+      <x:c r="A17" s="47" t="str">
         <x:v>iii_spl_diploma</x:v>
       </x:c>
-      <x:c r="B17" s="43" t="str">
+      <x:c r="B17" s="47" t="str">
         <x:v>compulsory</x:v>
       </x:c>
-      <x:c r="C17" s="43" t="str">
+      <x:c r="C17" s="47" t="str">
         <x:v>Compulsory</x:v>
       </x:c>
-      <x:c r="D17" s="43" t="str">
+      <x:c r="D17" s="47" t="str">
         <x:v>Approved InsureGPTE programme section.</x:v>
       </x:c>
-      <x:c r="E17" s="43"/>
-      <x:c r="F17" s="43"/>
-      <x:c r="G17" s="43" t="n">
+      <x:c r="E17" s="47"/>
+      <x:c r="F17" s="47"/>
+      <x:c r="G17" s="47" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H17" s="44" t="b">
+      <x:c r="H17" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="43" t="str">
+      <x:c r="A18" s="47" t="str">
         <x:v>iii_spl_diploma</x:v>
       </x:c>
-      <x:c r="B18" s="43" t="str">
+      <x:c r="B18" s="47" t="str">
         <x:v>spl_diploma</x:v>
       </x:c>
-      <x:c r="C18" s="43" t="str">
+      <x:c r="C18" s="47" t="str">
         <x:v>Spl_Diploma</x:v>
       </x:c>
-      <x:c r="D18" s="43" t="str">
+      <x:c r="D18" s="47" t="str">
         <x:v>Approved InsureGPTE programme section.</x:v>
       </x:c>
-      <x:c r="E18" s="43"/>
-      <x:c r="F18" s="43"/>
-      <x:c r="G18" s="43" t="n">
+      <x:c r="E18" s="47"/>
+      <x:c r="F18" s="47"/>
+      <x:c r="G18" s="47" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="H18" s="44" t="b">
+      <x:c r="H18" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="43" t="str">
+      <x:c r="A19" s="47" t="str">
         <x:v>iii_surveyor</x:v>
       </x:c>
-      <x:c r="B19" s="43" t="str">
+      <x:c r="B19" s="47" t="str">
         <x:v>compulsory</x:v>
       </x:c>
-      <x:c r="C19" s="43" t="str">
+      <x:c r="C19" s="47" t="str">
         <x:v>Compulsory</x:v>
       </x:c>
-      <x:c r="D19" s="43" t="str">
+      <x:c r="D19" s="47" t="str">
         <x:v>Approved InsureGPTE programme section.</x:v>
       </x:c>
-      <x:c r="E19" s="43"/>
-      <x:c r="F19" s="43"/>
-      <x:c r="G19" s="43" t="n">
+      <x:c r="E19" s="47"/>
+      <x:c r="F19" s="47"/>
+      <x:c r="G19" s="47" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H19" s="44" t="b">
+      <x:c r="H19" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="43" t="str">
+      <x:c r="A20" s="47" t="str">
         <x:v>iii_surveyor</x:v>
       </x:c>
-      <x:c r="B20" s="43" t="str">
+      <x:c r="B20" s="47" t="str">
         <x:v>surveyor</x:v>
       </x:c>
-      <x:c r="C20" s="43" t="str">
+      <x:c r="C20" s="47" t="str">
         <x:v>Surveyor</x:v>
       </x:c>
-      <x:c r="D20" s="43" t="str">
+      <x:c r="D20" s="47" t="str">
         <x:v>Approved InsureGPTE programme section.</x:v>
       </x:c>
-      <x:c r="E20" s="43"/>
-      <x:c r="F20" s="43"/>
-      <x:c r="G20" s="43" t="n">
+      <x:c r="E20" s="47"/>
+      <x:c r="F20" s="47"/>
+      <x:c r="G20" s="47" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="H20" s="44" t="b">
+      <x:c r="H20" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="43" t="str">
+      <x:c r="A21" s="47" t="str">
         <x:v>nia_direct_general_health</x:v>
       </x:c>
-      <x:c r="B21" s="43" t="str">
+      <x:c r="B21" s="47" t="str">
         <x:v>compulsory</x:v>
       </x:c>
-      <x:c r="C21" s="43" t="str">
+      <x:c r="C21" s="47" t="str">
         <x:v>Compulsory</x:v>
       </x:c>
-      <x:c r="D21" s="43" t="str">
+      <x:c r="D21" s="47" t="str">
         <x:v>Approved InsureGPTE programme section.</x:v>
       </x:c>
-      <x:c r="E21" s="43"/>
-      <x:c r="F21" s="43"/>
-      <x:c r="G21" s="43" t="n">
+      <x:c r="E21" s="47"/>
+      <x:c r="F21" s="47"/>
+      <x:c r="G21" s="47" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H21" s="44" t="b">
+      <x:c r="H21" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="43" t="str">
+      <x:c r="A22" s="47" t="str">
         <x:v>nia_direct_general_health</x:v>
       </x:c>
-      <x:c r="B22" s="43" t="str">
+      <x:c r="B22" s="47" t="str">
         <x:v>general_insurance</x:v>
       </x:c>
-      <x:c r="C22" s="43" t="str">
+      <x:c r="C22" s="47" t="str">
         <x:v>General Insurance</x:v>
       </x:c>
-      <x:c r="D22" s="43" t="str">
+      <x:c r="D22" s="47" t="str">
         <x:v>Approved InsureGPTE programme section.</x:v>
       </x:c>
-      <x:c r="E22" s="43"/>
-      <x:c r="F22" s="43"/>
-      <x:c r="G22" s="43" t="n">
+      <x:c r="E22" s="47"/>
+      <x:c r="F22" s="47"/>
+      <x:c r="G22" s="47" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="H22" s="44" t="b">
+      <x:c r="H22" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="43" t="str">
+      <x:c r="A23" s="47" t="str">
         <x:v>nia_direct_general_health</x:v>
       </x:c>
-      <x:c r="B23" s="43" t="str">
+      <x:c r="B23" s="47" t="str">
         <x:v>life_insurance</x:v>
       </x:c>
-      <x:c r="C23" s="43" t="str">
+      <x:c r="C23" s="47" t="str">
         <x:v>Life Insurance</x:v>
       </x:c>
-      <x:c r="D23" s="43" t="str">
+      <x:c r="D23" s="47" t="str">
         <x:v>Approved InsureGPTE programme section.</x:v>
       </x:c>
-      <x:c r="E23" s="43"/>
-      <x:c r="F23" s="43"/>
-      <x:c r="G23" s="43" t="n">
+      <x:c r="E23" s="47"/>
+      <x:c r="F23" s="47"/>
+      <x:c r="G23" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="H23" s="44" t="b">
+      <x:c r="H23" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="43" t="str">
+      <x:c r="A24" s="47" t="str">
         <x:v>nia_direct_general_health</x:v>
       </x:c>
-      <x:c r="B24" s="43" t="str">
+      <x:c r="B24" s="47" t="str">
         <x:v>broker</x:v>
       </x:c>
-      <x:c r="C24" s="43" t="str">
+      <x:c r="C24" s="47" t="str">
         <x:v>Broker</x:v>
       </x:c>
-      <x:c r="D24" s="43" t="str">
+      <x:c r="D24" s="47" t="str">
         <x:v>Approved InsureGPTE programme section.</x:v>
       </x:c>
-      <x:c r="E24" s="43"/>
-      <x:c r="F24" s="43"/>
-      <x:c r="G24" s="43" t="n">
+      <x:c r="E24" s="47"/>
+      <x:c r="F24" s="47"/>
+      <x:c r="G24" s="47" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="H24" s="44" t="b">
+      <x:c r="H24" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="43" t="str">
+      <x:c r="A25" s="47" t="str">
         <x:v>nia_reinsurance_broker</x:v>
       </x:c>
-      <x:c r="B25" s="43" t="str">
+      <x:c r="B25" s="47" t="str">
         <x:v>compulsory</x:v>
       </x:c>
-      <x:c r="C25" s="43" t="str">
+      <x:c r="C25" s="47" t="str">
         <x:v>Compulsory</x:v>
       </x:c>
-      <x:c r="D25" s="43" t="str">
+      <x:c r="D25" s="47" t="str">
         <x:v>Approved InsureGPTE programme section.</x:v>
       </x:c>
-      <x:c r="E25" s="43"/>
-      <x:c r="F25" s="43"/>
-      <x:c r="G25" s="43" t="n">
+      <x:c r="E25" s="47"/>
+      <x:c r="F25" s="47"/>
+      <x:c r="G25" s="47" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H25" s="44" t="b">
+      <x:c r="H25" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="43" t="str">
+      <x:c r="A26" s="47" t="str">
         <x:v>nia_reinsurance_broker</x:v>
       </x:c>
-      <x:c r="B26" s="43" t="str">
+      <x:c r="B26" s="47" t="str">
         <x:v>reinsurance</x:v>
       </x:c>
-      <x:c r="C26" s="43" t="str">
+      <x:c r="C26" s="47" t="str">
         <x:v>Reinsurance</x:v>
       </x:c>
-      <x:c r="D26" s="43" t="str">
+      <x:c r="D26" s="47" t="str">
         <x:v>Approved InsureGPTE programme section.</x:v>
       </x:c>
-      <x:c r="E26" s="43"/>
-      <x:c r="F26" s="43"/>
-      <x:c r="G26" s="43" t="n">
+      <x:c r="E26" s="47"/>
+      <x:c r="F26" s="47"/>
+      <x:c r="G26" s="47" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="H26" s="44" t="b">
+      <x:c r="H26" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="43" t="str">
+      <x:c r="A27" s="47" t="str">
         <x:v>nia_reinsurance_broker</x:v>
       </x:c>
-      <x:c r="B27" s="43" t="str">
+      <x:c r="B27" s="47" t="str">
         <x:v>broker</x:v>
       </x:c>
-      <x:c r="C27" s="43" t="str">
+      <x:c r="C27" s="47" t="str">
         <x:v>Broker</x:v>
       </x:c>
-      <x:c r="D27" s="43" t="str">
+      <x:c r="D27" s="47" t="str">
         <x:v>Approved InsureGPTE programme section.</x:v>
       </x:c>
-      <x:c r="E27" s="43"/>
-      <x:c r="F27" s="43"/>
-      <x:c r="G27" s="43" t="n">
+      <x:c r="E27" s="47"/>
+      <x:c r="F27" s="47"/>
+      <x:c r="G27" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="H27" s="44" t="b">
+      <x:c r="H27" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="43" t="str">
+      <x:c r="A28" s="47" t="str">
         <x:v>nia_composite_broker</x:v>
       </x:c>
-      <x:c r="B28" s="43" t="str">
+      <x:c r="B28" s="47" t="str">
         <x:v>compulsory</x:v>
       </x:c>
-      <x:c r="C28" s="43" t="str">
+      <x:c r="C28" s="47" t="str">
         <x:v>Compulsory</x:v>
       </x:c>
-      <x:c r="D28" s="43" t="str">
+      <x:c r="D28" s="47" t="str">
         <x:v>Approved InsureGPTE programme section.</x:v>
       </x:c>
-      <x:c r="E28" s="43"/>
-      <x:c r="F28" s="43"/>
-      <x:c r="G28" s="43" t="n">
+      <x:c r="E28" s="47"/>
+      <x:c r="F28" s="47"/>
+      <x:c r="G28" s="47" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="H28" s="44" t="b">
+      <x:c r="H28" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="43" t="str">
+      <x:c r="A29" s="47" t="str">
         <x:v>nia_composite_broker</x:v>
       </x:c>
-      <x:c r="B29" s="43" t="str">
+      <x:c r="B29" s="47" t="str">
         <x:v>general_insurance</x:v>
       </x:c>
-      <x:c r="C29" s="43" t="str">
+      <x:c r="C29" s="47" t="str">
         <x:v>General Insurance</x:v>
       </x:c>
-      <x:c r="D29" s="43" t="str">
+      <x:c r="D29" s="47" t="str">
         <x:v>Approved InsureGPTE programme section.</x:v>
       </x:c>
-      <x:c r="E29" s="43"/>
-      <x:c r="F29" s="43"/>
-      <x:c r="G29" s="43" t="n">
+      <x:c r="E29" s="47"/>
+      <x:c r="F29" s="47"/>
+      <x:c r="G29" s="47" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="H29" s="44" t="b">
+      <x:c r="H29" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="43" t="str">
+      <x:c r="A30" s="47" t="str">
         <x:v>nia_composite_broker</x:v>
       </x:c>
-      <x:c r="B30" s="43" t="str">
+      <x:c r="B30" s="47" t="str">
         <x:v>life_insurance</x:v>
       </x:c>
-      <x:c r="C30" s="43" t="str">
+      <x:c r="C30" s="47" t="str">
         <x:v>Life Insurance</x:v>
       </x:c>
-      <x:c r="D30" s="43" t="str">
+      <x:c r="D30" s="47" t="str">
         <x:v>Approved InsureGPTE programme section.</x:v>
       </x:c>
-      <x:c r="E30" s="43"/>
-      <x:c r="F30" s="43"/>
-      <x:c r="G30" s="43" t="n">
+      <x:c r="E30" s="47"/>
+      <x:c r="F30" s="47"/>
+      <x:c r="G30" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="H30" s="44" t="b">
+      <x:c r="H30" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="43" t="str">
+      <x:c r="A31" s="47" t="str">
         <x:v>nia_composite_broker</x:v>
       </x:c>
-      <x:c r="B31" s="43" t="str">
+      <x:c r="B31" s="47" t="str">
         <x:v>reinsurance</x:v>
       </x:c>
-      <x:c r="C31" s="43" t="str">
+      <x:c r="C31" s="47" t="str">
         <x:v>Reinsurance</x:v>
       </x:c>
-      <x:c r="D31" s="43" t="str">
+      <x:c r="D31" s="47" t="str">
         <x:v>Approved InsureGPTE programme section.</x:v>
       </x:c>
-      <x:c r="E31" s="43"/>
-      <x:c r="F31" s="43"/>
-      <x:c r="G31" s="43" t="n">
+      <x:c r="E31" s="47"/>
+      <x:c r="F31" s="47"/>
+      <x:c r="G31" s="47" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="H31" s="44" t="b">
+      <x:c r="H31" s="48" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="45" t="str">
+      <x:c r="A32" s="49" t="str">
         <x:v>nia_composite_broker</x:v>
       </x:c>
-      <x:c r="B32" s="45" t="str">
+      <x:c r="B32" s="49" t="str">
         <x:v>broker</x:v>
       </x:c>
-      <x:c r="C32" s="45" t="str">
+      <x:c r="C32" s="49" t="str">
         <x:v>Broker</x:v>
       </x:c>
-      <x:c r="D32" s="45" t="str">
+      <x:c r="D32" s="49" t="str">
         <x:v>Approved InsureGPTE programme section.</x:v>
       </x:c>
-      <x:c r="E32" s="45"/>
-      <x:c r="F32" s="45"/>
-      <x:c r="G32" s="45" t="n">
+      <x:c r="E32" s="49"/>
+      <x:c r="F32" s="49"/>
+      <x:c r="G32" s="49" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="H32" s="46" t="b">
+      <x:c r="H32" s="50" t="b">
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -46384,7 +46411,7 @@
     <x:dataValidation type="list" sqref="O2:O251">
       <x:formula1>"true,false"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" allowBlank="1" showDropDown="0" sqref="H2:H251">
+    <x:dataValidation type="list" errorStyle="stop" allowBlank="1" showDropDown="0" showErrorMessage="1" errorTitle="Invalid subject category" error="Choose one of the four approved Architecture Version 1.6 categories." sqref="H2:H251">
       <x:formula1>"General Insurance,Life Insurance,Common (Life &amp; Non-Life),Regulation and Compliance"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>

</xml_diff>